<commit_message>
update total column for pivot table
</commit_message>
<xml_diff>
--- a/misc/desk_review_template.xlsx
+++ b/misc/desk_review_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damajor\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CCAODATA\tmp\2026 Desk Review Workbooks Missing Sales\res_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8080567A-2060-4788-A3DF-CE1883463FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D870BD8A-0ADB-47B1-B291-14AD08489EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PIN Detail" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Neighborhood Breakout" sheetId="9" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="pin_detail_range">'PIN Detail'!$A$6:$BM$7</definedName>
+    <definedName name="pin_detail_range">'PIN Detail'!$A$6:$BL$7</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
@@ -266,21 +266,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BE6" authorId="0" shapeId="0" xr:uid="{9B95BB78-BBFA-4D08-898D-42D9F801F5C9}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Indicates that the PIN has homeownership improvement exemptions that have recently expired, implying that characteristics will be changed this tax year. 
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BF6" authorId="0" shapeId="0" xr:uid="{23361704-B7DC-4593-A117-F2816AD735D7}">
+    <comment ref="BE6" authorId="0" shapeId="0" xr:uid="{23361704-B7DC-4593-A117-F2816AD735D7}">
       <text>
         <r>
           <rPr>
@@ -293,7 +279,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BG6" authorId="0" shapeId="0" xr:uid="{AE640F8D-C8FE-48E7-A609-B0C718186353}">
+    <comment ref="BF6" authorId="0" shapeId="0" xr:uid="{AE640F8D-C8FE-48E7-A609-B0C718186353}">
       <text>
         <r>
           <rPr>
@@ -306,7 +292,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BH6" authorId="0" shapeId="0" xr:uid="{83117FFA-9BB4-4818-B2C6-422A3A943BE2}">
+    <comment ref="BG6" authorId="0" shapeId="0" xr:uid="{83117FFA-9BB4-4818-B2C6-422A3A943BE2}">
       <text>
         <r>
           <rPr>
@@ -319,7 +305,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BI6" authorId="0" shapeId="0" xr:uid="{66E115B5-8547-42A9-A19E-183D9317F2A3}">
+    <comment ref="BH6" authorId="0" shapeId="0" xr:uid="{66E115B5-8547-42A9-A19E-183D9317F2A3}">
       <text>
         <r>
           <rPr>
@@ -332,7 +318,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BJ6" authorId="0" shapeId="0" xr:uid="{C26E7A69-3354-428E-BBFF-70904DE96781}">
+    <comment ref="BI6" authorId="0" shapeId="0" xr:uid="{C26E7A69-3354-428E-BBFF-70904DE96781}">
       <text>
         <r>
           <rPr>
@@ -345,7 +331,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BK6" authorId="0" shapeId="0" xr:uid="{ACF72B43-181F-4EDF-AB31-F37EC8467982}">
+    <comment ref="BJ6" authorId="0" shapeId="0" xr:uid="{ACF72B43-181F-4EDF-AB31-F37EC8467982}">
       <text>
         <r>
           <rPr>
@@ -399,7 +385,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="87">
   <si>
     <t>Run ID (res):</t>
   </si>
@@ -534,9 +520,6 @@
   </si>
   <si>
     <t>Land Value Capped</t>
-  </si>
-  <si>
-    <t># Expired 288s</t>
   </si>
   <si>
     <t>Value Unchanged</t>
@@ -938,7 +921,7 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1084,6 +1067,7 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1092,7 +1076,19 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="114">
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
@@ -1106,10 +1102,304 @@
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
@@ -1149,11 +1439,11 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Damon Major" refreshedDate="46070.626223148145" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{2A499168-87FA-4E81-AAAC-57B5294536D8}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Damon Major" refreshedDate="46225.673710763891" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{2A499168-87FA-4E81-AAAC-57B5294536D8}">
   <cacheSource type="worksheet">
     <worksheetSource name="pin_detail_Range"/>
   </cacheSource>
-  <cacheFields count="65">
+  <cacheFields count="64">
     <cacheField name="PIN" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
@@ -1324,9 +1614,6 @@
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="Land Value Capped" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="# Expired 288s" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="Value Unchanged" numFmtId="0">
@@ -1429,7 +1716,6 @@
     <m/>
     <m/>
     <m/>
-    <m/>
   </r>
 </pivotCacheRecords>
 </file>
@@ -1437,7 +1723,7 @@
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D354C13E-180D-4071-9586-5999D6819012}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:G5" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="65">
+  <pivotFields count="64">
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
       <items count="2">
@@ -1459,6 +1745,19 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -1472,46 +1771,32 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
   </pivotFields>
   <rowFields count="2">
@@ -1551,80 +1836,98 @@
   </colItems>
   <dataFields count="6">
     <dataField name="Count of Class" fld="1" subtotal="count" baseField="2" baseItem="0" numFmtId="1"/>
-    <dataField name="Min of Total MV" fld="11" subtotal="min" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Average of Total MV" fld="11" subtotal="average" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Max of Total MV" fld="11" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Max of MV Difference" fld="64" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Min of Total MV" fld="62" subtotal="min" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Average of Total MV" fld="62" subtotal="average" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Max of Total MV" fld="62" subtotal="max" baseField="2" baseItem="0"/>
+    <dataField name="Max of MV Difference" fld="63" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
     <dataField name="Average of YoY ∆ %" fld="24" subtotal="average" baseField="2" baseItem="0" numFmtId="165"/>
   </dataFields>
-  <formats count="6">
-    <format dxfId="11">
+  <formats count="10">
+    <format dxfId="113">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4" selected="0">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1" selected="0">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="112">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="111">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4" selected="0">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1" selected="0">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="110">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="31">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4" selected="0">
+          <reference field="4294967294" count="1" selected="0">
             <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="29">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="17">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
             <x v="2"/>
-            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="15">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="3">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="6">
+    <format dxfId="1">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1">
             <x v="4"/>
           </reference>
         </references>
@@ -1940,58 +2243,58 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BM9"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:BL9"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="1" max="1" width="15.375" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="11.5" customWidth="1"/>
-    <col min="4" max="4" width="38.83203125" customWidth="1"/>
-    <col min="5" max="6" width="14.33203125" customWidth="1"/>
-    <col min="7" max="7" width="8.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.33203125" customWidth="1"/>
-    <col min="9" max="9" width="13.83203125" style="11" customWidth="1"/>
-    <col min="10" max="11" width="11.83203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.875" customWidth="1"/>
+    <col min="5" max="6" width="14.375" customWidth="1"/>
+    <col min="7" max="7" width="8.875" customWidth="1"/>
+    <col min="8" max="8" width="15.375" customWidth="1"/>
+    <col min="9" max="9" width="13.875" style="11" customWidth="1"/>
+    <col min="10" max="11" width="11.875" style="10" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13" style="10" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" style="10" customWidth="1"/>
-    <col min="14" max="14" width="10.58203125" style="10" customWidth="1"/>
-    <col min="15" max="15" width="9.08203125" style="11" customWidth="1"/>
-    <col min="16" max="16" width="13.58203125" style="15" customWidth="1"/>
-    <col min="17" max="18" width="11.58203125" style="10" customWidth="1"/>
-    <col min="19" max="19" width="13.58203125" style="10" customWidth="1"/>
+    <col min="13" max="13" width="10.875" style="10" customWidth="1"/>
+    <col min="14" max="14" width="10.625" style="10" customWidth="1"/>
+    <col min="15" max="15" width="9.125" style="11" customWidth="1"/>
+    <col min="16" max="16" width="13.625" style="15" customWidth="1"/>
+    <col min="17" max="18" width="11.625" style="10" customWidth="1"/>
+    <col min="19" max="19" width="13.625" style="10" customWidth="1"/>
     <col min="20" max="20" width="11" style="10"/>
-    <col min="21" max="21" width="10.83203125" style="10" customWidth="1"/>
-    <col min="22" max="22" width="11.08203125" style="10" customWidth="1"/>
-    <col min="23" max="23" width="11.58203125" style="11" customWidth="1"/>
+    <col min="21" max="21" width="10.875" style="10" customWidth="1"/>
+    <col min="22" max="22" width="11.125" style="10" customWidth="1"/>
+    <col min="23" max="23" width="11.625" style="11" customWidth="1"/>
     <col min="24" max="24" width="11" style="12"/>
     <col min="25" max="26" width="11" style="11"/>
-    <col min="27" max="27" width="21.08203125" style="11" customWidth="1"/>
+    <col min="27" max="27" width="21.125" style="11" customWidth="1"/>
     <col min="28" max="28" width="13" customWidth="1"/>
     <col min="29" max="29" width="13" style="10" customWidth="1"/>
-    <col min="30" max="30" width="18.58203125" style="10" customWidth="1"/>
+    <col min="30" max="30" width="18.625" style="10" customWidth="1"/>
     <col min="31" max="32" width="13" style="16" customWidth="1"/>
     <col min="33" max="33" width="13" style="10" customWidth="1"/>
-    <col min="34" max="34" width="18.58203125" style="10" customWidth="1"/>
+    <col min="34" max="34" width="18.625" style="10" customWidth="1"/>
     <col min="35" max="35" width="13" style="16" customWidth="1"/>
     <col min="37" max="37" width="9.25" customWidth="1"/>
-    <col min="38" max="38" width="7.33203125" customWidth="1"/>
-    <col min="40" max="40" width="15.08203125" customWidth="1"/>
-    <col min="41" max="41" width="15.58203125" customWidth="1"/>
-    <col min="42" max="42" width="15.33203125" customWidth="1"/>
-    <col min="44" max="44" width="8.08203125" customWidth="1"/>
+    <col min="38" max="38" width="7.375" customWidth="1"/>
+    <col min="40" max="40" width="15.125" customWidth="1"/>
+    <col min="41" max="41" width="15.625" customWidth="1"/>
+    <col min="42" max="42" width="15.375" customWidth="1"/>
+    <col min="44" max="44" width="8.125" customWidth="1"/>
     <col min="45" max="47" width="11" style="13"/>
     <col min="48" max="48" width="16" style="13" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="14" customWidth="1"/>
-    <col min="59" max="59" width="12.33203125" customWidth="1"/>
-    <col min="60" max="60" width="11.83203125" customWidth="1"/>
-    <col min="61" max="61" width="10.83203125" customWidth="1"/>
-    <col min="62" max="62" width="11.5" customWidth="1"/>
-    <col min="63" max="63" width="10" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="7.75" hidden="1" customWidth="1"/>
-    <col min="65" max="65" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="57" max="57" width="14" customWidth="1"/>
+    <col min="58" max="58" width="12.375" customWidth="1"/>
+    <col min="59" max="59" width="11.875" customWidth="1"/>
+    <col min="60" max="60" width="10.875" customWidth="1"/>
+    <col min="61" max="61" width="11.5" customWidth="1"/>
+    <col min="62" max="62" width="10" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="7.75" hidden="1" customWidth="1"/>
+    <col min="64" max="64" width="9.375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:65" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:64" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="5"/>
       <c r="B1" s="35"/>
       <c r="C1" s="35"/>
@@ -2054,9 +2357,8 @@
       <c r="BH1" s="5"/>
       <c r="BI1" s="5"/>
       <c r="BJ1" s="5"/>
-      <c r="BK1" s="5"/>
     </row>
-    <row r="2" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2096,7 +2398,7 @@
       <c r="AU2"/>
       <c r="AV2"/>
     </row>
-    <row r="3" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:64" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -2137,7 +2439,7 @@
       <c r="AU3"/>
       <c r="AV3"/>
     </row>
-    <row r="4" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:64" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="I4"/>
       <c r="J4"/>
@@ -2179,9 +2481,9 @@
       <c r="AU4" s="19"/>
       <c r="AV4"/>
     </row>
-    <row r="5" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:64" x14ac:dyDescent="0.25">
       <c r="B5" s="48" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C5" s="49"/>
       <c r="D5" s="49"/>
@@ -2205,15 +2507,15 @@
       <c r="V5" s="42"/>
       <c r="W5" s="43"/>
       <c r="X5" s="53" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Y5" s="54"/>
       <c r="Z5" s="55"/>
       <c r="AA5" s="23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AB5" s="44" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AC5" s="45"/>
       <c r="AD5" s="45"/>
@@ -2237,7 +2539,7 @@
       <c r="AT5" s="52"/>
       <c r="AU5" s="52"/>
       <c r="AV5" s="30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AW5" s="39" t="s">
         <v>2</v>
@@ -2254,10 +2556,9 @@
       <c r="BG5" s="40"/>
       <c r="BH5" s="40"/>
       <c r="BI5" s="40"/>
-      <c r="BJ5" s="40"/>
-      <c r="BK5" s="29"/>
+      <c r="BJ5" s="29"/>
     </row>
-    <row r="6" spans="1:65" ht="62" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:64" ht="63" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -2334,10 +2635,10 @@
         <v>24</v>
       </c>
       <c r="Z6" s="27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AA6" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AB6" s="2" t="s">
         <v>25</v>
@@ -2367,22 +2668,22 @@
         <v>33</v>
       </c>
       <c r="AK6" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="AL6" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="AL6" s="6" t="s">
+      <c r="AM6" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="AN6" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="AO6" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="AP6" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="AM6" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="AN6" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="AO6" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="AP6" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="AQ6" s="6" t="s">
         <v>34</v>
@@ -2400,16 +2701,16 @@
         <v>38</v>
       </c>
       <c r="AV6" s="22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AW6" s="9" t="s">
         <v>39</v>
       </c>
       <c r="AX6" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY6" s="9" t="s">
         <v>78</v>
-      </c>
-      <c r="AY6" s="9" t="s">
-        <v>79</v>
       </c>
       <c r="AZ6" s="9" t="s">
         <v>40</v>
@@ -2438,26 +2739,23 @@
       <c r="BH6" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="BI6" s="9" t="s">
+      <c r="BI6" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="BJ6" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="BK6" s="27" t="s">
-        <v>77</v>
-      </c>
-      <c r="BL6" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="BM6" s="4" t="s">
+      <c r="BJ6" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="BK6" s="3" t="s">
         <v>81</v>
       </c>
+      <c r="BL6" s="4" t="s">
+        <v>80</v>
+      </c>
     </row>
-    <row r="8" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:64" x14ac:dyDescent="0.25">
       <c r="AV8" s="17"/>
     </row>
-    <row r="9" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:64" x14ac:dyDescent="0.25">
       <c r="AV9" s="17"/>
     </row>
   </sheetData>
@@ -2465,7 +2763,7 @@
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="B1:J1"/>
     <mergeCell ref="J5:O5"/>
-    <mergeCell ref="AW5:BJ5"/>
+    <mergeCell ref="AW5:BI5"/>
     <mergeCell ref="P5:W5"/>
     <mergeCell ref="AB5:AI5"/>
     <mergeCell ref="B5:I5"/>
@@ -2481,27 +2779,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z4"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="1" max="1" width="15.375" customWidth="1"/>
     <col min="2" max="2" width="7.5" customWidth="1"/>
-    <col min="3" max="3" width="9.83203125" customWidth="1"/>
+    <col min="3" max="3" width="9.875" customWidth="1"/>
     <col min="4" max="4" width="10.5" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" style="15" customWidth="1"/>
-    <col min="6" max="7" width="14.58203125" style="10" customWidth="1"/>
+    <col min="5" max="5" width="11.875" style="15" customWidth="1"/>
+    <col min="6" max="7" width="14.625" style="10" customWidth="1"/>
     <col min="9" max="9" width="9.25" customWidth="1"/>
     <col min="10" max="10" width="15.5" customWidth="1"/>
     <col min="11" max="11" width="13.75" customWidth="1"/>
-    <col min="12" max="12" width="15.58203125" customWidth="1"/>
-    <col min="13" max="13" width="14.08203125" customWidth="1"/>
+    <col min="12" max="12" width="15.625" customWidth="1"/>
+    <col min="13" max="13" width="14.125" customWidth="1"/>
     <col min="14" max="14" width="15.75" customWidth="1"/>
     <col min="16" max="16" width="11" customWidth="1"/>
     <col min="17" max="17" width="11" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.35">
       <c r="B1" s="35" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C1" s="35"/>
       <c r="D1" s="35"/>
@@ -2528,7 +2826,7 @@
       <c r="Y1" s="5"/>
       <c r="Z1" s="5"/>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2538,9 +2836,9 @@
       <c r="G2"/>
       <c r="Q2"/>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B3" s="48" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C3" s="49"/>
       <c r="D3" s="50"/>
@@ -2548,7 +2846,7 @@
       <c r="F3" s="42"/>
       <c r="G3" s="43"/>
       <c r="H3" s="51" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I3" s="52"/>
       <c r="J3" s="52"/>
@@ -2562,12 +2860,12 @@
       <c r="R3" s="52"/>
       <c r="S3" s="56"/>
     </row>
-    <row r="4" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:26" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>4</v>
@@ -2576,37 +2874,37 @@
         <v>5</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>54</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>55</v>
       </c>
       <c r="H4" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="K4" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="N4" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="K4" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="N4" s="6" t="s">
+      <c r="O4" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>59</v>
       </c>
       <c r="P4" s="6" t="s">
         <v>35</v>
@@ -2637,68 +2935,69 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D773A1D3-FC14-4EA4-B569-35CAE3B3E4FA}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.58203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" style="33" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.9140625" style="33" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" style="33" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.25" style="33" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.9140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.875" style="33" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.625" style="33" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.125" style="33" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.625" style="33" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="B1" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C1" s="31"/>
       <c r="D1" s="31"/>
       <c r="E1" s="31"/>
       <c r="F1" s="31"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="E3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F3" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="B3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C3" s="32" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="32" t="s">
-        <v>86</v>
-      </c>
-      <c r="E3" s="32" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" s="32" t="s">
-        <v>84</v>
-      </c>
-      <c r="G3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="21" t="s">
-        <v>68</v>
-      </c>
       <c r="B4" s="26"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="57"/>
       <c r="F4" s="32"/>
       <c r="G4" s="25"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B5" s="26"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="57"/>
       <c r="F5" s="32"/>
       <c r="G5" s="25"/>
     </row>

</xml_diff>

<commit_message>
rename municipality name columns
</commit_message>
<xml_diff>
--- a/misc/desk_review_template.xlsx
+++ b/misc/desk_review_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CCAODATA\tmp\2026 Desk Review Workbooks Missing Sales\res_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D870BD8A-0ADB-47B1-B291-14AD08489EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{983178FC-DBB3-4FD4-8381-7D8723E6B02F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PIN Detail" sheetId="2" r:id="rId1"/>
@@ -921,7 +921,7 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1067,7 +1067,6 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1076,24 +1075,24 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
-  <dxfs count="114">
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+  <dxfs count="116">
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
@@ -1102,40 +1101,40 @@
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
@@ -1144,40 +1143,40 @@
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
@@ -1186,34 +1185,40 @@
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
@@ -1222,34 +1227,40 @@
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
@@ -1258,34 +1269,40 @@
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
@@ -1294,34 +1311,34 @@
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
@@ -1336,22 +1353,22 @@
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
@@ -1366,16 +1383,34 @@
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
@@ -1384,40 +1419,10 @@
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1439,7 +1444,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Damon Major" refreshedDate="46225.673710763891" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{2A499168-87FA-4E81-AAAC-57B5294536D8}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Damon Major" refreshedDate="46225.817303935182" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{2A499168-87FA-4E81-AAAC-57B5294536D8}">
   <cacheSource type="worksheet">
     <worksheetSource name="pin_detail_Range"/>
   </cacheSource>
@@ -1838,11 +1843,29 @@
     <dataField name="Count of Class" fld="1" subtotal="count" baseField="2" baseItem="0" numFmtId="1"/>
     <dataField name="Min of Total MV" fld="62" subtotal="min" baseField="2" baseItem="0" numFmtId="164"/>
     <dataField name="Average of Total MV" fld="62" subtotal="average" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Max of Total MV" fld="62" subtotal="max" baseField="2" baseItem="0"/>
+    <dataField name="Max of Total MV" fld="62" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
     <dataField name="Max of MV Difference" fld="63" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
     <dataField name="Average of YoY ∆ %" fld="24" subtotal="average" baseField="2" baseItem="0" numFmtId="165"/>
   </dataFields>
-  <formats count="10">
+  <formats count="12">
+    <format dxfId="115">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="114">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
     <format dxfId="113">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
@@ -1865,7 +1888,7 @@
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
-            <x v="4"/>
+            <x v="1"/>
           </reference>
         </references>
       </pivotArea>
@@ -1874,30 +1897,12 @@
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
-            <x v="4"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="31">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
             <x v="1"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="29">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="17">
+    <format dxfId="109">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -1906,7 +1911,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="15">
+    <format dxfId="108">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -1915,7 +1920,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="3">
+    <format dxfId="107">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -1924,11 +1929,29 @@
         </references>
       </pivotArea>
     </format>
+    <format dxfId="106">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="3">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
     <format dxfId="1">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
-            <x v="4"/>
+            <x v="3"/>
           </reference>
         </references>
       </pivotArea>
@@ -2244,57 +2267,57 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BL9"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.375" customWidth="1"/>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="11.5" customWidth="1"/>
-    <col min="4" max="4" width="38.875" customWidth="1"/>
-    <col min="5" max="6" width="14.375" customWidth="1"/>
-    <col min="7" max="7" width="8.875" customWidth="1"/>
-    <col min="8" max="8" width="15.375" customWidth="1"/>
-    <col min="9" max="9" width="13.875" style="11" customWidth="1"/>
-    <col min="10" max="11" width="11.875" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.83203125" customWidth="1"/>
+    <col min="5" max="6" width="14.33203125" customWidth="1"/>
+    <col min="7" max="7" width="8.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.33203125" customWidth="1"/>
+    <col min="9" max="9" width="13.83203125" style="11" customWidth="1"/>
+    <col min="10" max="11" width="11.83203125" style="10" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13" style="10" customWidth="1"/>
-    <col min="13" max="13" width="10.875" style="10" customWidth="1"/>
-    <col min="14" max="14" width="10.625" style="10" customWidth="1"/>
-    <col min="15" max="15" width="9.125" style="11" customWidth="1"/>
-    <col min="16" max="16" width="13.625" style="15" customWidth="1"/>
-    <col min="17" max="18" width="11.625" style="10" customWidth="1"/>
-    <col min="19" max="19" width="13.625" style="10" customWidth="1"/>
+    <col min="13" max="13" width="10.83203125" style="10" customWidth="1"/>
+    <col min="14" max="14" width="10.58203125" style="10" customWidth="1"/>
+    <col min="15" max="15" width="9.08203125" style="11" customWidth="1"/>
+    <col min="16" max="16" width="13.58203125" style="15" customWidth="1"/>
+    <col min="17" max="18" width="11.58203125" style="10" customWidth="1"/>
+    <col min="19" max="19" width="13.58203125" style="10" customWidth="1"/>
     <col min="20" max="20" width="11" style="10"/>
-    <col min="21" max="21" width="10.875" style="10" customWidth="1"/>
-    <col min="22" max="22" width="11.125" style="10" customWidth="1"/>
-    <col min="23" max="23" width="11.625" style="11" customWidth="1"/>
+    <col min="21" max="21" width="10.83203125" style="10" customWidth="1"/>
+    <col min="22" max="22" width="11.08203125" style="10" customWidth="1"/>
+    <col min="23" max="23" width="11.58203125" style="11" customWidth="1"/>
     <col min="24" max="24" width="11" style="12"/>
     <col min="25" max="26" width="11" style="11"/>
-    <col min="27" max="27" width="21.125" style="11" customWidth="1"/>
+    <col min="27" max="27" width="21.08203125" style="11" customWidth="1"/>
     <col min="28" max="28" width="13" customWidth="1"/>
     <col min="29" max="29" width="13" style="10" customWidth="1"/>
-    <col min="30" max="30" width="18.625" style="10" customWidth="1"/>
+    <col min="30" max="30" width="18.58203125" style="10" customWidth="1"/>
     <col min="31" max="32" width="13" style="16" customWidth="1"/>
     <col min="33" max="33" width="13" style="10" customWidth="1"/>
-    <col min="34" max="34" width="18.625" style="10" customWidth="1"/>
+    <col min="34" max="34" width="18.58203125" style="10" customWidth="1"/>
     <col min="35" max="35" width="13" style="16" customWidth="1"/>
     <col min="37" max="37" width="9.25" customWidth="1"/>
-    <col min="38" max="38" width="7.375" customWidth="1"/>
-    <col min="40" max="40" width="15.125" customWidth="1"/>
-    <col min="41" max="41" width="15.625" customWidth="1"/>
-    <col min="42" max="42" width="15.375" customWidth="1"/>
-    <col min="44" max="44" width="8.125" customWidth="1"/>
+    <col min="38" max="38" width="7.33203125" customWidth="1"/>
+    <col min="40" max="40" width="15.08203125" customWidth="1"/>
+    <col min="41" max="41" width="15.58203125" customWidth="1"/>
+    <col min="42" max="42" width="15.33203125" customWidth="1"/>
+    <col min="44" max="44" width="8.08203125" customWidth="1"/>
     <col min="45" max="47" width="11" style="13"/>
     <col min="48" max="48" width="16" style="13" bestFit="1" customWidth="1"/>
     <col min="57" max="57" width="14" customWidth="1"/>
-    <col min="58" max="58" width="12.375" customWidth="1"/>
-    <col min="59" max="59" width="11.875" customWidth="1"/>
-    <col min="60" max="60" width="10.875" customWidth="1"/>
+    <col min="58" max="58" width="12.33203125" customWidth="1"/>
+    <col min="59" max="59" width="11.83203125" customWidth="1"/>
+    <col min="60" max="60" width="10.83203125" customWidth="1"/>
     <col min="61" max="61" width="11.5" customWidth="1"/>
     <col min="62" max="62" width="10" bestFit="1" customWidth="1"/>
     <col min="63" max="63" width="7.75" hidden="1" customWidth="1"/>
-    <col min="64" max="64" width="9.375" hidden="1" customWidth="1"/>
+    <col min="64" max="64" width="9.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:64" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:64" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="5"/>
       <c r="B1" s="35"/>
       <c r="C1" s="35"/>
@@ -2358,7 +2381,7 @@
       <c r="BI1" s="5"/>
       <c r="BJ1" s="5"/>
     </row>
-    <row r="2" spans="1:64" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:64" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2398,7 +2421,7 @@
       <c r="AU2"/>
       <c r="AV2"/>
     </row>
-    <row r="3" spans="1:64" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:64" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -2439,7 +2462,7 @@
       <c r="AU3"/>
       <c r="AV3"/>
     </row>
-    <row r="4" spans="1:64" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:64" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="I4"/>
       <c r="J4"/>
@@ -2481,7 +2504,7 @@
       <c r="AU4" s="19"/>
       <c r="AV4"/>
     </row>
-    <row r="5" spans="1:64" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:64" x14ac:dyDescent="0.35">
       <c r="B5" s="48" t="s">
         <v>59</v>
       </c>
@@ -2558,7 +2581,7 @@
       <c r="BI5" s="40"/>
       <c r="BJ5" s="29"/>
     </row>
-    <row r="6" spans="1:64" ht="63" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:64" ht="62" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -2752,10 +2775,10 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:64" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:64" x14ac:dyDescent="0.35">
       <c r="AV8" s="17"/>
     </row>
-    <row r="9" spans="1:64" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:64" x14ac:dyDescent="0.35">
       <c r="AV9" s="17"/>
     </row>
   </sheetData>
@@ -2779,25 +2802,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z4"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.375" customWidth="1"/>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="7.5" customWidth="1"/>
-    <col min="3" max="3" width="9.875" customWidth="1"/>
+    <col min="3" max="3" width="9.83203125" customWidth="1"/>
     <col min="4" max="4" width="10.5" customWidth="1"/>
-    <col min="5" max="5" width="11.875" style="15" customWidth="1"/>
-    <col min="6" max="7" width="14.625" style="10" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" style="15" customWidth="1"/>
+    <col min="6" max="7" width="14.58203125" style="10" customWidth="1"/>
     <col min="9" max="9" width="9.25" customWidth="1"/>
     <col min="10" max="10" width="15.5" customWidth="1"/>
     <col min="11" max="11" width="13.75" customWidth="1"/>
-    <col min="12" max="12" width="15.625" customWidth="1"/>
-    <col min="13" max="13" width="14.125" customWidth="1"/>
+    <col min="12" max="12" width="15.58203125" customWidth="1"/>
+    <col min="13" max="13" width="14.08203125" customWidth="1"/>
     <col min="14" max="14" width="15.75" customWidth="1"/>
     <col min="16" max="16" width="11" customWidth="1"/>
     <col min="17" max="17" width="11" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.5">
       <c r="B1" s="35" t="s">
         <v>50</v>
       </c>
@@ -2826,7 +2849,7 @@
       <c r="Y1" s="5"/>
       <c r="Z1" s="5"/>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2836,7 +2859,7 @@
       <c r="G2"/>
       <c r="Q2"/>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="B3" s="48" t="s">
         <v>61</v>
       </c>
@@ -2860,7 +2883,7 @@
       <c r="R3" s="52"/>
       <c r="S3" s="56"/>
     </row>
-    <row r="4" spans="1:26" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>3</v>
       </c>
@@ -2935,19 +2958,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D773A1D3-FC14-4EA4-B569-35CAE3B3E4FA}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.875" style="33" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.625" style="33" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.125" style="33" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.625" style="33" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.58203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" style="33" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.9140625" style="33" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" style="33" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.25" style="33" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.9140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.5">
       <c r="B1" s="5" t="s">
         <v>69</v>
       </c>
@@ -2956,7 +2979,7 @@
       <c r="E1" s="31"/>
       <c r="F1" s="31"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="24" t="s">
         <v>66</v>
       </c>
@@ -2969,7 +2992,7 @@
       <c r="D3" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="12" t="s">
         <v>84</v>
       </c>
       <c r="F3" s="32" t="s">
@@ -2979,25 +3002,25 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="21" t="s">
         <v>67</v>
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="12"/>
       <c r="D4" s="12"/>
-      <c r="E4" s="57"/>
+      <c r="E4" s="12"/>
       <c r="F4" s="32"/>
       <c r="G4" s="25"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="21" t="s">
         <v>68</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
-      <c r="E5" s="57"/>
+      <c r="E5" s="12"/>
       <c r="F5" s="32"/>
       <c r="G5" s="25"/>
     </row>

</xml_diff>

<commit_message>
replace desk review template
</commit_message>
<xml_diff>
--- a/misc/desk_review_template.xlsx
+++ b/misc/desk_review_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damajor\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CCAODATA\tmp\2026 Desk Review Workbooks Missing Sales\res_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8080567A-2060-4788-A3DF-CE1883463FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{983178FC-DBB3-4FD4-8381-7D8723E6B02F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PIN Detail" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Neighborhood Breakout" sheetId="9" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="pin_detail_range">'PIN Detail'!$A$6:$BM$7</definedName>
+    <definedName name="pin_detail_range">'PIN Detail'!$A$6:$BL$7</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
@@ -266,21 +266,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BE6" authorId="0" shapeId="0" xr:uid="{9B95BB78-BBFA-4D08-898D-42D9F801F5C9}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Indicates that the PIN has homeownership improvement exemptions that have recently expired, implying that characteristics will be changed this tax year. 
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BF6" authorId="0" shapeId="0" xr:uid="{23361704-B7DC-4593-A117-F2816AD735D7}">
+    <comment ref="BE6" authorId="0" shapeId="0" xr:uid="{23361704-B7DC-4593-A117-F2816AD735D7}">
       <text>
         <r>
           <rPr>
@@ -293,7 +279,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BG6" authorId="0" shapeId="0" xr:uid="{AE640F8D-C8FE-48E7-A609-B0C718186353}">
+    <comment ref="BF6" authorId="0" shapeId="0" xr:uid="{AE640F8D-C8FE-48E7-A609-B0C718186353}">
       <text>
         <r>
           <rPr>
@@ -306,7 +292,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BH6" authorId="0" shapeId="0" xr:uid="{83117FFA-9BB4-4818-B2C6-422A3A943BE2}">
+    <comment ref="BG6" authorId="0" shapeId="0" xr:uid="{83117FFA-9BB4-4818-B2C6-422A3A943BE2}">
       <text>
         <r>
           <rPr>
@@ -319,7 +305,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BI6" authorId="0" shapeId="0" xr:uid="{66E115B5-8547-42A9-A19E-183D9317F2A3}">
+    <comment ref="BH6" authorId="0" shapeId="0" xr:uid="{66E115B5-8547-42A9-A19E-183D9317F2A3}">
       <text>
         <r>
           <rPr>
@@ -332,7 +318,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BJ6" authorId="0" shapeId="0" xr:uid="{C26E7A69-3354-428E-BBFF-70904DE96781}">
+    <comment ref="BI6" authorId="0" shapeId="0" xr:uid="{C26E7A69-3354-428E-BBFF-70904DE96781}">
       <text>
         <r>
           <rPr>
@@ -345,7 +331,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BK6" authorId="0" shapeId="0" xr:uid="{ACF72B43-181F-4EDF-AB31-F37EC8467982}">
+    <comment ref="BJ6" authorId="0" shapeId="0" xr:uid="{ACF72B43-181F-4EDF-AB31-F37EC8467982}">
       <text>
         <r>
           <rPr>
@@ -399,7 +385,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="87">
   <si>
     <t>Run ID (res):</t>
   </si>
@@ -534,9 +520,6 @@
   </si>
   <si>
     <t>Land Value Capped</t>
-  </si>
-  <si>
-    <t># Expired 288s</t>
   </si>
   <si>
     <t>Value Unchanged</t>
@@ -1092,12 +1075,24 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+  <dxfs count="116">
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
@@ -1118,16 +1113,316 @@
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1149,11 +1444,11 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Damon Major" refreshedDate="46070.626223148145" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{2A499168-87FA-4E81-AAAC-57B5294536D8}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Damon Major" refreshedDate="46225.817303935182" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{2A499168-87FA-4E81-AAAC-57B5294536D8}">
   <cacheSource type="worksheet">
     <worksheetSource name="pin_detail_Range"/>
   </cacheSource>
-  <cacheFields count="65">
+  <cacheFields count="64">
     <cacheField name="PIN" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
@@ -1324,9 +1619,6 @@
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="Land Value Capped" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="# Expired 288s" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="Value Unchanged" numFmtId="0">
@@ -1429,7 +1721,6 @@
     <m/>
     <m/>
     <m/>
-    <m/>
   </r>
 </pivotCacheRecords>
 </file>
@@ -1437,7 +1728,7 @@
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D354C13E-180D-4071-9586-5999D6819012}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:G5" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="65">
+  <pivotFields count="64">
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
       <items count="2">
@@ -1459,6 +1750,19 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -1472,46 +1776,32 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
   </pivotFields>
   <rowFields count="2">
@@ -1551,81 +1841,117 @@
   </colItems>
   <dataFields count="6">
     <dataField name="Count of Class" fld="1" subtotal="count" baseField="2" baseItem="0" numFmtId="1"/>
-    <dataField name="Min of Total MV" fld="11" subtotal="min" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Average of Total MV" fld="11" subtotal="average" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Max of Total MV" fld="11" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Max of MV Difference" fld="64" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Min of Total MV" fld="62" subtotal="min" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Average of Total MV" fld="62" subtotal="average" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Max of Total MV" fld="62" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Max of MV Difference" fld="63" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
     <dataField name="Average of YoY ∆ %" fld="24" subtotal="average" baseField="2" baseItem="0" numFmtId="165"/>
   </dataFields>
-  <formats count="6">
-    <format dxfId="11">
+  <formats count="12">
+    <format dxfId="115">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4" selected="0">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1" selected="0">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="114">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="113">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4" selected="0">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1" selected="0">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="112">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="111">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4" selected="0">
+          <reference field="4294967294" count="1" selected="0">
             <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="110">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="109">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
             <x v="2"/>
-            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="108">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="107">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="6">
+    <format dxfId="106">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="1"/>
-            <x v="2"/>
+          <reference field="4294967294" count="1">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="3">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
             <x v="3"/>
-            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="3"/>
           </reference>
         </references>
       </pivotArea>
@@ -1940,7 +2266,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BM9"/>
+  <dimension ref="A1:BL9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
@@ -1981,17 +2307,17 @@
     <col min="44" max="44" width="8.08203125" customWidth="1"/>
     <col min="45" max="47" width="11" style="13"/>
     <col min="48" max="48" width="16" style="13" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="14" customWidth="1"/>
-    <col min="59" max="59" width="12.33203125" customWidth="1"/>
-    <col min="60" max="60" width="11.83203125" customWidth="1"/>
-    <col min="61" max="61" width="10.83203125" customWidth="1"/>
-    <col min="62" max="62" width="11.5" customWidth="1"/>
-    <col min="63" max="63" width="10" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="7.75" hidden="1" customWidth="1"/>
-    <col min="65" max="65" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="57" max="57" width="14" customWidth="1"/>
+    <col min="58" max="58" width="12.33203125" customWidth="1"/>
+    <col min="59" max="59" width="11.83203125" customWidth="1"/>
+    <col min="60" max="60" width="10.83203125" customWidth="1"/>
+    <col min="61" max="61" width="11.5" customWidth="1"/>
+    <col min="62" max="62" width="10" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="7.75" hidden="1" customWidth="1"/>
+    <col min="64" max="64" width="9.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:65" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:64" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="5"/>
       <c r="B1" s="35"/>
       <c r="C1" s="35"/>
@@ -2054,9 +2380,8 @@
       <c r="BH1" s="5"/>
       <c r="BI1" s="5"/>
       <c r="BJ1" s="5"/>
-      <c r="BK1" s="5"/>
     </row>
-    <row r="2" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:64" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2096,7 +2421,7 @@
       <c r="AU2"/>
       <c r="AV2"/>
     </row>
-    <row r="3" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:64" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -2137,7 +2462,7 @@
       <c r="AU3"/>
       <c r="AV3"/>
     </row>
-    <row r="4" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:64" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="I4"/>
       <c r="J4"/>
@@ -2179,9 +2504,9 @@
       <c r="AU4" s="19"/>
       <c r="AV4"/>
     </row>
-    <row r="5" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:64" x14ac:dyDescent="0.35">
       <c r="B5" s="48" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C5" s="49"/>
       <c r="D5" s="49"/>
@@ -2205,15 +2530,15 @@
       <c r="V5" s="42"/>
       <c r="W5" s="43"/>
       <c r="X5" s="53" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Y5" s="54"/>
       <c r="Z5" s="55"/>
       <c r="AA5" s="23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AB5" s="44" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AC5" s="45"/>
       <c r="AD5" s="45"/>
@@ -2237,7 +2562,7 @@
       <c r="AT5" s="52"/>
       <c r="AU5" s="52"/>
       <c r="AV5" s="30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AW5" s="39" t="s">
         <v>2</v>
@@ -2254,10 +2579,9 @@
       <c r="BG5" s="40"/>
       <c r="BH5" s="40"/>
       <c r="BI5" s="40"/>
-      <c r="BJ5" s="40"/>
-      <c r="BK5" s="29"/>
+      <c r="BJ5" s="29"/>
     </row>
-    <row r="6" spans="1:65" ht="62" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:64" ht="62" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -2334,10 +2658,10 @@
         <v>24</v>
       </c>
       <c r="Z6" s="27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AA6" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AB6" s="2" t="s">
         <v>25</v>
@@ -2367,22 +2691,22 @@
         <v>33</v>
       </c>
       <c r="AK6" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="AL6" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="AL6" s="6" t="s">
+      <c r="AM6" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="AN6" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="AO6" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="AP6" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="AM6" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="AN6" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="AO6" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="AP6" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="AQ6" s="6" t="s">
         <v>34</v>
@@ -2400,16 +2724,16 @@
         <v>38</v>
       </c>
       <c r="AV6" s="22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AW6" s="9" t="s">
         <v>39</v>
       </c>
       <c r="AX6" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY6" s="9" t="s">
         <v>78</v>
-      </c>
-      <c r="AY6" s="9" t="s">
-        <v>79</v>
       </c>
       <c r="AZ6" s="9" t="s">
         <v>40</v>
@@ -2438,26 +2762,23 @@
       <c r="BH6" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="BI6" s="9" t="s">
+      <c r="BI6" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="BJ6" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="BK6" s="27" t="s">
-        <v>77</v>
-      </c>
-      <c r="BL6" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="BM6" s="4" t="s">
+      <c r="BJ6" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="BK6" s="3" t="s">
         <v>81</v>
       </c>
+      <c r="BL6" s="4" t="s">
+        <v>80</v>
+      </c>
     </row>
-    <row r="8" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:64" x14ac:dyDescent="0.35">
       <c r="AV8" s="17"/>
     </row>
-    <row r="9" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:64" x14ac:dyDescent="0.35">
       <c r="AV9" s="17"/>
     </row>
   </sheetData>
@@ -2465,7 +2786,7 @@
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="B1:J1"/>
     <mergeCell ref="J5:O5"/>
-    <mergeCell ref="AW5:BJ5"/>
+    <mergeCell ref="AW5:BI5"/>
     <mergeCell ref="P5:W5"/>
     <mergeCell ref="AB5:AI5"/>
     <mergeCell ref="B5:I5"/>
@@ -2501,7 +2822,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.5">
       <c r="B1" s="35" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C1" s="35"/>
       <c r="D1" s="35"/>
@@ -2540,7 +2861,7 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="B3" s="48" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C3" s="49"/>
       <c r="D3" s="50"/>
@@ -2548,7 +2869,7 @@
       <c r="F3" s="42"/>
       <c r="G3" s="43"/>
       <c r="H3" s="51" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I3" s="52"/>
       <c r="J3" s="52"/>
@@ -2567,7 +2888,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>4</v>
@@ -2576,37 +2897,37 @@
         <v>5</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>54</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>55</v>
       </c>
       <c r="H4" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="K4" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="N4" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="K4" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="N4" s="6" t="s">
+      <c r="O4" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>59</v>
       </c>
       <c r="P4" s="6" t="s">
         <v>35</v>
@@ -2646,11 +2967,12 @@
     <col min="5" max="5" width="14.6640625" style="33" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.25" style="33" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.9140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.5">
       <c r="B1" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C1" s="31"/>
       <c r="D1" s="31"/>
@@ -2659,46 +2981,46 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="F3" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" t="s">
         <v>71</v>
-      </c>
-      <c r="C3" s="32" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="32" t="s">
-        <v>86</v>
-      </c>
-      <c r="E3" s="32" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" s="32" t="s">
-        <v>84</v>
-      </c>
-      <c r="G3" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B4" s="26"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
       <c r="F4" s="32"/>
       <c r="G4" s="25"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B5" s="26"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
       <c r="F5" s="32"/>
       <c r="G5" s="25"/>
     </row>

</xml_diff>

<commit_message>
include updates to changes from outside PR
</commit_message>
<xml_diff>
--- a/misc/desk_review_template.xlsx
+++ b/misc/desk_review_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damajor\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CCAODATA\tmp\2026 Desk Review Workbooks Missing Sales\res_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8080567A-2060-4788-A3DF-CE1883463FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{983178FC-DBB3-4FD4-8381-7D8723E6B02F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PIN Detail" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Neighborhood Breakout" sheetId="9" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="pin_detail_range">'PIN Detail'!$A$6:$BM$7</definedName>
+    <definedName name="pin_detail_range">'PIN Detail'!$A$6:$BL$7</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
@@ -266,21 +266,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BE6" authorId="0" shapeId="0" xr:uid="{9B95BB78-BBFA-4D08-898D-42D9F801F5C9}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Indicates that the PIN has homeownership improvement exemptions that have recently expired, implying that characteristics will be changed this tax year. 
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BF6" authorId="0" shapeId="0" xr:uid="{23361704-B7DC-4593-A117-F2816AD735D7}">
+    <comment ref="BE6" authorId="0" shapeId="0" xr:uid="{23361704-B7DC-4593-A117-F2816AD735D7}">
       <text>
         <r>
           <rPr>
@@ -293,7 +279,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BG6" authorId="0" shapeId="0" xr:uid="{AE640F8D-C8FE-48E7-A609-B0C718186353}">
+    <comment ref="BF6" authorId="0" shapeId="0" xr:uid="{AE640F8D-C8FE-48E7-A609-B0C718186353}">
       <text>
         <r>
           <rPr>
@@ -306,7 +292,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BH6" authorId="0" shapeId="0" xr:uid="{83117FFA-9BB4-4818-B2C6-422A3A943BE2}">
+    <comment ref="BG6" authorId="0" shapeId="0" xr:uid="{83117FFA-9BB4-4818-B2C6-422A3A943BE2}">
       <text>
         <r>
           <rPr>
@@ -319,7 +305,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BI6" authorId="0" shapeId="0" xr:uid="{66E115B5-8547-42A9-A19E-183D9317F2A3}">
+    <comment ref="BH6" authorId="0" shapeId="0" xr:uid="{66E115B5-8547-42A9-A19E-183D9317F2A3}">
       <text>
         <r>
           <rPr>
@@ -332,7 +318,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BJ6" authorId="0" shapeId="0" xr:uid="{C26E7A69-3354-428E-BBFF-70904DE96781}">
+    <comment ref="BI6" authorId="0" shapeId="0" xr:uid="{C26E7A69-3354-428E-BBFF-70904DE96781}">
       <text>
         <r>
           <rPr>
@@ -345,7 +331,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BK6" authorId="0" shapeId="0" xr:uid="{ACF72B43-181F-4EDF-AB31-F37EC8467982}">
+    <comment ref="BJ6" authorId="0" shapeId="0" xr:uid="{ACF72B43-181F-4EDF-AB31-F37EC8467982}">
       <text>
         <r>
           <rPr>
@@ -399,7 +385,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="87">
   <si>
     <t>Run ID (res):</t>
   </si>
@@ -534,9 +520,6 @@
   </si>
   <si>
     <t>Land Value Capped</t>
-  </si>
-  <si>
-    <t># Expired 288s</t>
   </si>
   <si>
     <t>Value Unchanged</t>
@@ -1092,12 +1075,24 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+  <dxfs count="116">
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
@@ -1118,16 +1113,316 @@
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1149,11 +1444,11 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Damon Major" refreshedDate="46070.626223148145" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{2A499168-87FA-4E81-AAAC-57B5294536D8}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Damon Major" refreshedDate="46225.817303935182" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{2A499168-87FA-4E81-AAAC-57B5294536D8}">
   <cacheSource type="worksheet">
     <worksheetSource name="pin_detail_Range"/>
   </cacheSource>
-  <cacheFields count="65">
+  <cacheFields count="64">
     <cacheField name="PIN" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
@@ -1324,9 +1619,6 @@
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="Land Value Capped" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="# Expired 288s" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="Value Unchanged" numFmtId="0">
@@ -1429,7 +1721,6 @@
     <m/>
     <m/>
     <m/>
-    <m/>
   </r>
 </pivotCacheRecords>
 </file>
@@ -1437,7 +1728,7 @@
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D354C13E-180D-4071-9586-5999D6819012}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:G5" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="65">
+  <pivotFields count="64">
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
       <items count="2">
@@ -1459,6 +1750,19 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -1472,46 +1776,32 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
   </pivotFields>
   <rowFields count="2">
@@ -1551,81 +1841,117 @@
   </colItems>
   <dataFields count="6">
     <dataField name="Count of Class" fld="1" subtotal="count" baseField="2" baseItem="0" numFmtId="1"/>
-    <dataField name="Min of Total MV" fld="11" subtotal="min" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Average of Total MV" fld="11" subtotal="average" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Max of Total MV" fld="11" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Max of MV Difference" fld="64" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Min of Total MV" fld="62" subtotal="min" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Average of Total MV" fld="62" subtotal="average" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Max of Total MV" fld="62" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Max of MV Difference" fld="63" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
     <dataField name="Average of YoY ∆ %" fld="24" subtotal="average" baseField="2" baseItem="0" numFmtId="165"/>
   </dataFields>
-  <formats count="6">
-    <format dxfId="11">
+  <formats count="12">
+    <format dxfId="115">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4" selected="0">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1" selected="0">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="114">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="113">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4" selected="0">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1" selected="0">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="112">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="111">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4" selected="0">
+          <reference field="4294967294" count="1" selected="0">
             <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="110">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="109">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
             <x v="2"/>
-            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="108">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="107">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="6">
+    <format dxfId="106">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="1"/>
-            <x v="2"/>
+          <reference field="4294967294" count="1">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="3">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
             <x v="3"/>
-            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="3"/>
           </reference>
         </references>
       </pivotArea>
@@ -1940,7 +2266,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BM9"/>
+  <dimension ref="A1:BL9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
@@ -1981,17 +2307,17 @@
     <col min="44" max="44" width="8.08203125" customWidth="1"/>
     <col min="45" max="47" width="11" style="13"/>
     <col min="48" max="48" width="16" style="13" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="14" customWidth="1"/>
-    <col min="59" max="59" width="12.33203125" customWidth="1"/>
-    <col min="60" max="60" width="11.83203125" customWidth="1"/>
-    <col min="61" max="61" width="10.83203125" customWidth="1"/>
-    <col min="62" max="62" width="11.5" customWidth="1"/>
-    <col min="63" max="63" width="10" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="7.75" hidden="1" customWidth="1"/>
-    <col min="65" max="65" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="57" max="57" width="14" customWidth="1"/>
+    <col min="58" max="58" width="12.33203125" customWidth="1"/>
+    <col min="59" max="59" width="11.83203125" customWidth="1"/>
+    <col min="60" max="60" width="10.83203125" customWidth="1"/>
+    <col min="61" max="61" width="11.5" customWidth="1"/>
+    <col min="62" max="62" width="10" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="7.75" hidden="1" customWidth="1"/>
+    <col min="64" max="64" width="9.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:65" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:64" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="5"/>
       <c r="B1" s="35"/>
       <c r="C1" s="35"/>
@@ -2054,9 +2380,8 @@
       <c r="BH1" s="5"/>
       <c r="BI1" s="5"/>
       <c r="BJ1" s="5"/>
-      <c r="BK1" s="5"/>
     </row>
-    <row r="2" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:64" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2096,7 +2421,7 @@
       <c r="AU2"/>
       <c r="AV2"/>
     </row>
-    <row r="3" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:64" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -2137,7 +2462,7 @@
       <c r="AU3"/>
       <c r="AV3"/>
     </row>
-    <row r="4" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:64" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="I4"/>
       <c r="J4"/>
@@ -2179,9 +2504,9 @@
       <c r="AU4" s="19"/>
       <c r="AV4"/>
     </row>
-    <row r="5" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:64" x14ac:dyDescent="0.35">
       <c r="B5" s="48" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C5" s="49"/>
       <c r="D5" s="49"/>
@@ -2205,15 +2530,15 @@
       <c r="V5" s="42"/>
       <c r="W5" s="43"/>
       <c r="X5" s="53" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Y5" s="54"/>
       <c r="Z5" s="55"/>
       <c r="AA5" s="23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AB5" s="44" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AC5" s="45"/>
       <c r="AD5" s="45"/>
@@ -2237,7 +2562,7 @@
       <c r="AT5" s="52"/>
       <c r="AU5" s="52"/>
       <c r="AV5" s="30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AW5" s="39" t="s">
         <v>2</v>
@@ -2254,10 +2579,9 @@
       <c r="BG5" s="40"/>
       <c r="BH5" s="40"/>
       <c r="BI5" s="40"/>
-      <c r="BJ5" s="40"/>
-      <c r="BK5" s="29"/>
+      <c r="BJ5" s="29"/>
     </row>
-    <row r="6" spans="1:65" ht="62" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:64" ht="62" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -2334,10 +2658,10 @@
         <v>24</v>
       </c>
       <c r="Z6" s="27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AA6" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AB6" s="2" t="s">
         <v>25</v>
@@ -2367,22 +2691,22 @@
         <v>33</v>
       </c>
       <c r="AK6" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="AL6" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="AL6" s="6" t="s">
+      <c r="AM6" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="AN6" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="AO6" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="AP6" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="AM6" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="AN6" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="AO6" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="AP6" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="AQ6" s="6" t="s">
         <v>34</v>
@@ -2400,16 +2724,16 @@
         <v>38</v>
       </c>
       <c r="AV6" s="22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AW6" s="9" t="s">
         <v>39</v>
       </c>
       <c r="AX6" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY6" s="9" t="s">
         <v>78</v>
-      </c>
-      <c r="AY6" s="9" t="s">
-        <v>79</v>
       </c>
       <c r="AZ6" s="9" t="s">
         <v>40</v>
@@ -2438,26 +2762,23 @@
       <c r="BH6" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="BI6" s="9" t="s">
+      <c r="BI6" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="BJ6" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="BK6" s="27" t="s">
-        <v>77</v>
-      </c>
-      <c r="BL6" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="BM6" s="4" t="s">
+      <c r="BJ6" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="BK6" s="3" t="s">
         <v>81</v>
       </c>
+      <c r="BL6" s="4" t="s">
+        <v>80</v>
+      </c>
     </row>
-    <row r="8" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:64" x14ac:dyDescent="0.35">
       <c r="AV8" s="17"/>
     </row>
-    <row r="9" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:64" x14ac:dyDescent="0.35">
       <c r="AV9" s="17"/>
     </row>
   </sheetData>
@@ -2465,7 +2786,7 @@
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="B1:J1"/>
     <mergeCell ref="J5:O5"/>
-    <mergeCell ref="AW5:BJ5"/>
+    <mergeCell ref="AW5:BI5"/>
     <mergeCell ref="P5:W5"/>
     <mergeCell ref="AB5:AI5"/>
     <mergeCell ref="B5:I5"/>
@@ -2501,7 +2822,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.5">
       <c r="B1" s="35" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C1" s="35"/>
       <c r="D1" s="35"/>
@@ -2540,7 +2861,7 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="B3" s="48" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C3" s="49"/>
       <c r="D3" s="50"/>
@@ -2548,7 +2869,7 @@
       <c r="F3" s="42"/>
       <c r="G3" s="43"/>
       <c r="H3" s="51" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I3" s="52"/>
       <c r="J3" s="52"/>
@@ -2567,7 +2888,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>4</v>
@@ -2576,37 +2897,37 @@
         <v>5</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>54</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>55</v>
       </c>
       <c r="H4" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="K4" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="N4" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="K4" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="N4" s="6" t="s">
+      <c r="O4" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>59</v>
       </c>
       <c r="P4" s="6" t="s">
         <v>35</v>
@@ -2646,11 +2967,12 @@
     <col min="5" max="5" width="14.6640625" style="33" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.25" style="33" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.9140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.5">
       <c r="B1" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C1" s="31"/>
       <c r="D1" s="31"/>
@@ -2659,46 +2981,46 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="F3" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" t="s">
         <v>71</v>
-      </c>
-      <c r="C3" s="32" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="32" t="s">
-        <v>86</v>
-      </c>
-      <c r="E3" s="32" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" s="32" t="s">
-        <v>84</v>
-      </c>
-      <c r="G3" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B4" s="26"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
       <c r="F4" s="32"/>
       <c r="G4" s="25"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B5" s="26"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
       <c r="F5" s="32"/>
       <c r="G5" s="25"/>
     </row>

</xml_diff>

<commit_message>
Update desk review templates and municipality column name (#537)
This updates three things in the desk review workbooks
- switches `cook_municipality_name` to `tax_municipality name` since we
no longer have that column in model.assessment_pin
- removes the column `# Expired 288s`
- standardizes the pivot tables to use total_mv

lintr errors are from outside the scope of the issue.

---------

Co-authored-by: Jean Cochrane <jeancochrane@users.noreply.github.com>
Co-authored-by: Sweaty Handshake <william.ridgeway@cookcountyil.gov>
</commit_message>
<xml_diff>
--- a/misc/desk_review_template.xlsx
+++ b/misc/desk_review_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damajor\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\CCAODATA\tmp\2026 Desk Review Workbooks Missing Sales\res_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8080567A-2060-4788-A3DF-CE1883463FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{983178FC-DBB3-4FD4-8381-7D8723E6B02F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PIN Detail" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Neighborhood Breakout" sheetId="9" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="pin_detail_range">'PIN Detail'!$A$6:$BM$7</definedName>
+    <definedName name="pin_detail_range">'PIN Detail'!$A$6:$BL$7</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
@@ -266,21 +266,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BE6" authorId="0" shapeId="0" xr:uid="{9B95BB78-BBFA-4D08-898D-42D9F801F5C9}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Indicates that the PIN has homeownership improvement exemptions that have recently expired, implying that characteristics will be changed this tax year. 
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="BF6" authorId="0" shapeId="0" xr:uid="{23361704-B7DC-4593-A117-F2816AD735D7}">
+    <comment ref="BE6" authorId="0" shapeId="0" xr:uid="{23361704-B7DC-4593-A117-F2816AD735D7}">
       <text>
         <r>
           <rPr>
@@ -293,7 +279,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BG6" authorId="0" shapeId="0" xr:uid="{AE640F8D-C8FE-48E7-A609-B0C718186353}">
+    <comment ref="BF6" authorId="0" shapeId="0" xr:uid="{AE640F8D-C8FE-48E7-A609-B0C718186353}">
       <text>
         <r>
           <rPr>
@@ -306,7 +292,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BH6" authorId="0" shapeId="0" xr:uid="{83117FFA-9BB4-4818-B2C6-422A3A943BE2}">
+    <comment ref="BG6" authorId="0" shapeId="0" xr:uid="{83117FFA-9BB4-4818-B2C6-422A3A943BE2}">
       <text>
         <r>
           <rPr>
@@ -319,7 +305,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BI6" authorId="0" shapeId="0" xr:uid="{66E115B5-8547-42A9-A19E-183D9317F2A3}">
+    <comment ref="BH6" authorId="0" shapeId="0" xr:uid="{66E115B5-8547-42A9-A19E-183D9317F2A3}">
       <text>
         <r>
           <rPr>
@@ -332,7 +318,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BJ6" authorId="0" shapeId="0" xr:uid="{C26E7A69-3354-428E-BBFF-70904DE96781}">
+    <comment ref="BI6" authorId="0" shapeId="0" xr:uid="{C26E7A69-3354-428E-BBFF-70904DE96781}">
       <text>
         <r>
           <rPr>
@@ -345,7 +331,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BK6" authorId="0" shapeId="0" xr:uid="{ACF72B43-181F-4EDF-AB31-F37EC8467982}">
+    <comment ref="BJ6" authorId="0" shapeId="0" xr:uid="{ACF72B43-181F-4EDF-AB31-F37EC8467982}">
       <text>
         <r>
           <rPr>
@@ -399,7 +385,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="87">
   <si>
     <t>Run ID (res):</t>
   </si>
@@ -534,9 +520,6 @@
   </si>
   <si>
     <t>Land Value Capped</t>
-  </si>
-  <si>
-    <t># Expired 288s</t>
   </si>
   <si>
     <t>Value Unchanged</t>
@@ -1092,12 +1075,24 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+  <dxfs count="116">
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
@@ -1118,16 +1113,316 @@
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
       <alignment horizontal="right"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1149,11 +1444,11 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Damon Major" refreshedDate="46070.626223148145" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{2A499168-87FA-4E81-AAAC-57B5294536D8}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Damon Major" refreshedDate="46225.817303935182" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{2A499168-87FA-4E81-AAAC-57B5294536D8}">
   <cacheSource type="worksheet">
     <worksheetSource name="pin_detail_Range"/>
   </cacheSource>
-  <cacheFields count="65">
+  <cacheFields count="64">
     <cacheField name="PIN" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
@@ -1324,9 +1619,6 @@
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="Land Value Capped" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="# Expired 288s" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="Value Unchanged" numFmtId="0">
@@ -1429,7 +1721,6 @@
     <m/>
     <m/>
     <m/>
-    <m/>
   </r>
 </pivotCacheRecords>
 </file>
@@ -1437,7 +1728,7 @@
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D354C13E-180D-4071-9586-5999D6819012}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:G5" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="65">
+  <pivotFields count="64">
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
       <items count="2">
@@ -1459,6 +1750,19 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -1472,46 +1776,32 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
   </pivotFields>
   <rowFields count="2">
@@ -1551,81 +1841,117 @@
   </colItems>
   <dataFields count="6">
     <dataField name="Count of Class" fld="1" subtotal="count" baseField="2" baseItem="0" numFmtId="1"/>
-    <dataField name="Min of Total MV" fld="11" subtotal="min" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Average of Total MV" fld="11" subtotal="average" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Max of Total MV" fld="11" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
-    <dataField name="Max of MV Difference" fld="64" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Min of Total MV" fld="62" subtotal="min" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Average of Total MV" fld="62" subtotal="average" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Max of Total MV" fld="62" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
+    <dataField name="Max of MV Difference" fld="63" subtotal="max" baseField="2" baseItem="0" numFmtId="164"/>
     <dataField name="Average of YoY ∆ %" fld="24" subtotal="average" baseField="2" baseItem="0" numFmtId="165"/>
   </dataFields>
-  <formats count="6">
-    <format dxfId="11">
+  <formats count="12">
+    <format dxfId="115">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4" selected="0">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1" selected="0">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="114">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="113">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4" selected="0">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1" selected="0">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="112">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
+          <reference field="4294967294" count="1">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="111">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4" selected="0">
+          <reference field="4294967294" count="1" selected="0">
             <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="110">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="109">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
             <x v="2"/>
-            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="108">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="107">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="6">
+    <format dxfId="106">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="1"/>
-            <x v="2"/>
+          <reference field="4294967294" count="1">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="3">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
             <x v="3"/>
-            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="3"/>
           </reference>
         </references>
       </pivotArea>
@@ -1940,7 +2266,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BM9"/>
+  <dimension ref="A1:BL9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
@@ -1981,17 +2307,17 @@
     <col min="44" max="44" width="8.08203125" customWidth="1"/>
     <col min="45" max="47" width="11" style="13"/>
     <col min="48" max="48" width="16" style="13" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="14" customWidth="1"/>
-    <col min="59" max="59" width="12.33203125" customWidth="1"/>
-    <col min="60" max="60" width="11.83203125" customWidth="1"/>
-    <col min="61" max="61" width="10.83203125" customWidth="1"/>
-    <col min="62" max="62" width="11.5" customWidth="1"/>
-    <col min="63" max="63" width="10" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="7.75" hidden="1" customWidth="1"/>
-    <col min="65" max="65" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="57" max="57" width="14" customWidth="1"/>
+    <col min="58" max="58" width="12.33203125" customWidth="1"/>
+    <col min="59" max="59" width="11.83203125" customWidth="1"/>
+    <col min="60" max="60" width="10.83203125" customWidth="1"/>
+    <col min="61" max="61" width="11.5" customWidth="1"/>
+    <col min="62" max="62" width="10" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="7.75" hidden="1" customWidth="1"/>
+    <col min="64" max="64" width="9.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:65" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:64" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="5"/>
       <c r="B1" s="35"/>
       <c r="C1" s="35"/>
@@ -2054,9 +2380,8 @@
       <c r="BH1" s="5"/>
       <c r="BI1" s="5"/>
       <c r="BJ1" s="5"/>
-      <c r="BK1" s="5"/>
     </row>
-    <row r="2" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:64" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2096,7 +2421,7 @@
       <c r="AU2"/>
       <c r="AV2"/>
     </row>
-    <row r="3" spans="1:65" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:64" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -2137,7 +2462,7 @@
       <c r="AU3"/>
       <c r="AV3"/>
     </row>
-    <row r="4" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:64" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="I4"/>
       <c r="J4"/>
@@ -2179,9 +2504,9 @@
       <c r="AU4" s="19"/>
       <c r="AV4"/>
     </row>
-    <row r="5" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:64" x14ac:dyDescent="0.35">
       <c r="B5" s="48" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C5" s="49"/>
       <c r="D5" s="49"/>
@@ -2205,15 +2530,15 @@
       <c r="V5" s="42"/>
       <c r="W5" s="43"/>
       <c r="X5" s="53" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Y5" s="54"/>
       <c r="Z5" s="55"/>
       <c r="AA5" s="23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AB5" s="44" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AC5" s="45"/>
       <c r="AD5" s="45"/>
@@ -2237,7 +2562,7 @@
       <c r="AT5" s="52"/>
       <c r="AU5" s="52"/>
       <c r="AV5" s="30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AW5" s="39" t="s">
         <v>2</v>
@@ -2254,10 +2579,9 @@
       <c r="BG5" s="40"/>
       <c r="BH5" s="40"/>
       <c r="BI5" s="40"/>
-      <c r="BJ5" s="40"/>
-      <c r="BK5" s="29"/>
+      <c r="BJ5" s="29"/>
     </row>
-    <row r="6" spans="1:65" ht="62" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:64" ht="62" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -2334,10 +2658,10 @@
         <v>24</v>
       </c>
       <c r="Z6" s="27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="AA6" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AB6" s="2" t="s">
         <v>25</v>
@@ -2367,22 +2691,22 @@
         <v>33</v>
       </c>
       <c r="AK6" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="AL6" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="AL6" s="6" t="s">
+      <c r="AM6" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="AN6" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="AO6" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="AP6" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="AM6" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="AN6" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="AO6" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="AP6" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="AQ6" s="6" t="s">
         <v>34</v>
@@ -2400,16 +2724,16 @@
         <v>38</v>
       </c>
       <c r="AV6" s="22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AW6" s="9" t="s">
         <v>39</v>
       </c>
       <c r="AX6" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="AY6" s="9" t="s">
         <v>78</v>
-      </c>
-      <c r="AY6" s="9" t="s">
-        <v>79</v>
       </c>
       <c r="AZ6" s="9" t="s">
         <v>40</v>
@@ -2438,26 +2762,23 @@
       <c r="BH6" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="BI6" s="9" t="s">
+      <c r="BI6" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="BJ6" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="BK6" s="27" t="s">
-        <v>77</v>
-      </c>
-      <c r="BL6" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="BM6" s="4" t="s">
+      <c r="BJ6" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="BK6" s="3" t="s">
         <v>81</v>
       </c>
+      <c r="BL6" s="4" t="s">
+        <v>80</v>
+      </c>
     </row>
-    <row r="8" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:64" x14ac:dyDescent="0.35">
       <c r="AV8" s="17"/>
     </row>
-    <row r="9" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:64" x14ac:dyDescent="0.35">
       <c r="AV9" s="17"/>
     </row>
   </sheetData>
@@ -2465,7 +2786,7 @@
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="B1:J1"/>
     <mergeCell ref="J5:O5"/>
-    <mergeCell ref="AW5:BJ5"/>
+    <mergeCell ref="AW5:BI5"/>
     <mergeCell ref="P5:W5"/>
     <mergeCell ref="AB5:AI5"/>
     <mergeCell ref="B5:I5"/>
@@ -2501,7 +2822,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.5">
       <c r="B1" s="35" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C1" s="35"/>
       <c r="D1" s="35"/>
@@ -2540,7 +2861,7 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="B3" s="48" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C3" s="49"/>
       <c r="D3" s="50"/>
@@ -2548,7 +2869,7 @@
       <c r="F3" s="42"/>
       <c r="G3" s="43"/>
       <c r="H3" s="51" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I3" s="52"/>
       <c r="J3" s="52"/>
@@ -2567,7 +2888,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>4</v>
@@ -2576,37 +2897,37 @@
         <v>5</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>54</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>55</v>
       </c>
       <c r="H4" s="18" t="s">
         <v>33</v>
       </c>
       <c r="I4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="K4" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="N4" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="K4" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="N4" s="6" t="s">
+      <c r="O4" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>59</v>
       </c>
       <c r="P4" s="6" t="s">
         <v>35</v>
@@ -2646,11 +2967,12 @@
     <col min="5" max="5" width="14.6640625" style="33" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.25" style="33" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.9140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.5">
       <c r="B1" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C1" s="31"/>
       <c r="D1" s="31"/>
@@ -2659,46 +2981,46 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="F3" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" t="s">
         <v>71</v>
-      </c>
-      <c r="C3" s="32" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="32" t="s">
-        <v>86</v>
-      </c>
-      <c r="E3" s="32" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" s="32" t="s">
-        <v>84</v>
-      </c>
-      <c r="G3" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B4" s="26"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
       <c r="F4" s="32"/>
       <c r="G4" s="25"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B5" s="26"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
       <c r="F5" s="32"/>
       <c r="G5" s="25"/>
     </row>

</xml_diff>